<commit_message>
Replace players 17 and 18 with ATAL and REC Green Technologies and five sourced Hong Kong PV projects each
</commit_message>
<xml_diff>
--- a/market-research/hong-kong-solar/Hong_Kong_Solar_Market_Players.xlsx
+++ b/market-research/hong-kong-solar/Hong_Kong_Solar_Market_Players.xlsx
@@ -1210,84 +1210,84 @@
     <row r="18" ht="144" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Billion Smart Green Energy Limited（骏盈绿色能源）</t>
-        </is>
-      </c>
-      <c r="B18" s="7" t="inlineStr">
-        <is>
-          <t>未核实到公司官网URL</t>
+          <t>ATAL（安乐工程集团／Analogue Holdings Limited）</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>https://www.atal.com/</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>未找到可核实的具名太阳能项目。公司主体可由香港公司注册处及商标公报核实；未将台湾Billion Electric／Billion Watts的项目归入本公司。</t>
-        </is>
-      </c>
-      <c r="D18" s="7" t="inlineStr">
-        <is>
-          <t>未找到可核实的公开项目资料</t>
-        </is>
-      </c>
-      <c r="E18" s="7" t="inlineStr">
-        <is>
-          <t>未找到可核实的公开项目资料</t>
-        </is>
-      </c>
-      <c r="F18" s="7" t="inlineStr">
-        <is>
-          <t>未找到可核实的公开项目资料</t>
-        </is>
-      </c>
-      <c r="G18" s="7" t="inlineStr">
-        <is>
-          <t>未找到可核实的公开项目资料</t>
+          <t>香港科学园第二及第三期｜供应及安装太阳能光伏系统，并提供BMS及视听等智能楼宇系统；官网项目页列示；未披露光伏装机容量。</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>太古坊一座 One Taikoo Place｜提供太阳能光伏板及BMS、CCTV、ELV等智能绿色系统；官网项目页确认参与；光伏容量未披露。</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>如心园 Nina Park，荃湾｜参与可步行式太阳能光伏地砖系统安装；集团2023年ESG报告披露；未披露容量及独立完工日期。</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>AIRSIDE，启德｜参与太阳能光伏地砖系统安装；集团2023年ESG报告披露；属于光伏建筑一体化应用，容量及独立完工日期未披露。</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>利园三期 Lee Garden Three，铜锣湾｜参与太阳能光伏地砖系统安装；集团2023年ESG报告披露；未披露容量及独立完工日期。</t>
         </is>
       </c>
       <c r="H18" s="7" t="inlineStr">
         <is>
-          <t>未找到可核实的2025年或累计光伏总装机容量披露。</t>
+          <t>未找到可核实的2025年或累计光伏总装机容量披露；上述项目均为香港项目，未将集团其他机电工程规模计为光伏装机。</t>
         </is>
       </c>
     </row>
     <row r="19" ht="144" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>3Tech Engineering（3Tech）</t>
+          <t>REC Green Technologies Company Limited（RGT）</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>https://www.3tech.net/</t>
+          <t>https://www.rec-gt.com/</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>香港晨曦岛 Town Island 可再生能源项目｜公司官方沿革确认完成；属于光伏／可再生能源供电工程，获得香港工程项目奖；本来源未披露其具体合同容量。</t>
+          <t>石壁水塘漂浮式光伏系统｜官网确认安装，为附近抽水站供电，并列为香港首个漂浮式光伏系统；公司页面未披露容量及完工年份。</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>龙岩未来城数字经济产业园，中国福建｜交付光伏车棚＋充电桩混合系统；120块380 W组件、76.8 kWh磷酸铁锂储能；与国电通合作。</t>
+          <t>小蚝湾污水处理厂综合光伏示范系统｜安装可步行式、单晶硅及薄膜光伏组件；此为官网所述示范系统，未将全厂1.1 MW容量归给RGT。</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>阿曼电讯混合供电案例（客户／站点未具名）｜7.68 kW太阳能板，配柴油机及电池；公司产品册列为项目实绩，未列完工年份。</t>
+          <t>昂船洲污水处理厂｜官网确认参与CIGS铜铟镓硒薄膜光伏示范，并列渠务署为客户；未披露其具体容量及完工年份。</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>阿根廷混合供电案例（客户／站点未具名）｜公司册展示太阳能棚混合供电；1.2 kW为负载而非光伏装机，故不作为装机容量；未列年份。</t>
+          <t>葵涌基本污水处理厂｜展示智能组件、功率优化器与单晶硅光伏系统的比较应用；官网确认参与；未披露容量及年份。</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>北非主要电讯运营商离网站点计划｜客户需求覆盖逾1,000座电讯塔；2018年末招标，客户选用3Tech交钥匙光伏＋储能＋柴油方案；未披露实际交付站数及总光伏容量。</t>
+          <t>新田雨水泵房 San Tin Stormwater Pumping Station｜官网光伏项目列表列示，客户为渠务署；具体供货／承包范围、容量及年份未披露。</t>
         </is>
       </c>
       <c r="H19" s="6" t="inlineStr">
         <is>
-          <t>未找到可核实的2025年或累计光伏总装机容量披露。</t>
+          <t>未找到可核实的2025年或累计光伏总装机容量披露；官网列有香港光伏工程及示范项目，未提供公司整体MW／kW总量。</t>
         </is>
       </c>
     </row>
@@ -1468,17 +1468,22 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="rId89"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId90"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B19" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B21" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B18" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F18" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B19" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B21" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId107"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Replace players 16, 19 and 20 with JEC, Well Green and Solar Farm HK and sourced Hong Kong solar projects
</commit_message>
<xml_diff>
--- a/market-research/hong-kong-solar/Hong_Kong_Solar_Market_Players.xlsx
+++ b/market-research/hong-kong-solar/Hong_Kong_Solar_Market_Players.xlsx
@@ -1168,42 +1168,42 @@
     <row r="17" ht="144" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>XOLAREN GLOBAL（XOLAREN）</t>
+          <t>JEC（怡和机器／Jardine Engineering Corporation）</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>https://www.xolaren.com/</t>
+          <t>https://www.jec.com/</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Akij Polymer Industries／Akij Bashir集团，孟加拉｜2.01 MW屋顶光伏；官方帖文确认技术负责人为IDCOL贷款方独立工程师／顾问，完成COD检查；EPC为NetZero，并非XOLAREN。</t>
+          <t>启德体育园｜1 MWp太阳能光伏系统；公司2024可持续发展报告确认交付；此为该项目容量，非JEC累计装机。</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Hameem集团，孟加拉｜16.9 MW屋顶光伏；同名公开账号自述的技术负责人履历：贷款方独立工程师；未经客户佐证，非已确认公司EPC交付。</t>
+          <t>香港大学，薄扶林｜公司2024可持续发展报告确认已安装光伏解决方案；未披露具体楼名、容量及独立完工日期。</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>孟加拉工程技术大学 BUET（与PSL）｜3.27 MW屋顶光伏；同名公开账号自述的技术负责人顾问项目，未经客户佐证；未披露投运日期。</t>
+          <t>元朗净水设施第一阶段 Yuen Long Effluent Polishing Plant｜2022-07获渠务署机电工程合同，范围含光伏及3套热电联供机组；当时预计2026年完成，未据此认定光伏已投运；容量未披露。</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>TK集团／Samuda Green Energy，孟加拉｜2.4 MW工商业屋顶光伏；同名公开账号自述的技术负责人顾问项目，未经客户佐证；规划扩建至30 MW不计为已装。</t>
+          <t>赤鱲角消防局｜设计、供应及安装太阳能光伏系统；JEC 2019年第44期公司刊物列示；未披露装机容量及独立完工日期。</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>未找到第五个可核实的独立项目；官网客户标识未足以证明具体太阳能EPC合同。</t>
-        </is>
-      </c>
-      <c r="H17" s="5" t="inlineStr">
-        <is>
-          <t>约5 MW交付里程碑｜公司官方LinkedIn帖文称正在达到“5 MW of Solar Projects delivered across Bangladesh”；未给出精确统计截止日。地区为孟加拉，非香港装机，亦无2025年末更新总量；保留原文“reaching”的限定。</t>
+          <t>工业贸易大楼，启德｜太阳能光伏系统项目；JEC 2019年第44期公司刊物确认参与；未披露装机容量及独立完工日期。</t>
+        </is>
+      </c>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>未找到可核实的2025年或累计光伏总装机容量披露；下列单个项目容量不代表公司总装机。</t>
         </is>
       </c>
     </row>
@@ -1294,84 +1294,84 @@
     <row r="20" ht="144" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Theo Solar（目录对应：Theo Environmental Technology Co. Ltd.／天皓环境科技）</t>
+          <t>Well Green Energy Technology Co. Ltd.（威曜绿色能源科技）</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>https://www.theoenv.com/en/index.php</t>
+          <t>https://solar.wellgreen.com.hk/</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>未找到可核实的具名已实施太阳能项目；官网Case Studies页仅嵌入视频，未列客户、地点或容量；Smartflower产品展示不作为五个独立工程。</t>
-        </is>
-      </c>
-      <c r="D20" s="7" t="inlineStr">
-        <is>
-          <t>未找到可核实的公开项目资料</t>
-        </is>
-      </c>
-      <c r="E20" s="7" t="inlineStr">
-        <is>
-          <t>未找到可核实的公开项目资料</t>
-        </is>
-      </c>
-      <c r="F20" s="7" t="inlineStr">
-        <is>
-          <t>未找到可核实的公开项目资料</t>
-        </is>
-      </c>
-      <c r="G20" s="7" t="inlineStr">
-        <is>
-          <t>未找到可核实的公开项目资料</t>
-        </is>
-      </c>
-      <c r="H20" s="7" t="inlineStr">
-        <is>
-          <t>未找到可核实的2025年或累计光伏总装机容量披露。</t>
+          <t>香港中文大学晨兴书院｜官网重点项目标为2025年；太阳能系统工程；未披露装机容量及详细承包分工。</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>环保园 EcoPark｜200 kW、634块太阳能板；官网具名光伏案例；未列完工年份。</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>香港外展训练学校 Outward Bound｜139 kW、342块太阳能板；官网具名光伏案例；未列完工年份。</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>香港游乐场协会｜92.81 kW、258块太阳能板；官网确认规划天台光伏项目；未列独立完工年份。</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>职工盟培训中心 CTU｜42 kW、108块太阳能板；官网确认天台安装案例；未列完工年份。</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>未找到可核实的2025年或累计光伏总装机容量披露；下列单个项目容量不代表公司总装机。官网披露完成逾300个项目，但未给出对应MW／kW总量。</t>
         </is>
       </c>
     </row>
     <row r="21" ht="144" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Lik Kai Engineering Co., Ltd.（力佳工程）</t>
+          <t>Solar Farm HK Limited（太阳农庄）</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>https://www.likkai.com.hk/</t>
+          <t>https://solarfarm.com.hk/</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>未找到可核实的具名太阳能工程。机电工程署承办商名录可核实其光伏安装服务；未把新鸿基集团其他公司的光伏项目直接归给力佳。</t>
-        </is>
-      </c>
-      <c r="D21" s="6" t="inlineStr">
-        <is>
-          <t>未找到可核实的公开项目资料</t>
-        </is>
-      </c>
-      <c r="E21" s="6" t="inlineStr">
-        <is>
-          <t>未找到可核实的公开项目资料</t>
-        </is>
-      </c>
-      <c r="F21" s="6" t="inlineStr">
-        <is>
-          <t>未找到可核实的公开项目资料</t>
-        </is>
-      </c>
-      <c r="G21" s="6" t="inlineStr">
-        <is>
-          <t>未找到可核实的公开项目资料</t>
+          <t>中信银行国际，尖沙咀广东道旗舰分行｜BIPV太阳能玻璃外墙；官网列为实际案例；未披露装机容量及完工年份。</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>天水围 +WOO 嘉湖｜官网具名太阳能工程案例；具体承包范围、装机容量及完工年份未披露。</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>大埔运头塘商场｜官网具名太阳能案例；同一场址两组照片合并计一个项目；容量及完工年份未披露。</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>落马洲河套区创科园｜官网具名太阳能案例；未进一步披露楼座、合同分工、装机容量及完工年份。</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>赤鱲角商贸港物流中心 Tradeport｜官网具名太阳能案例；具体承包范围、容量及完工年份未披露。</t>
         </is>
       </c>
       <c r="H21" s="6" t="inlineStr">
         <is>
-          <t>未找到可核实的2025年或累计光伏总装机容量披露。</t>
+          <t>未找到可核实的2025年或累计光伏总装机容量披露；下列单个项目容量不代表公司总装机。</t>
         </is>
       </c>
     </row>
@@ -1467,23 +1467,31 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId88"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="rId89"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B18" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F18" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B19" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B21" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B18" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F18" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B19" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B21" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId115"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>